<commit_message>
data: add matched skincare catalog controls
</commit_message>
<xml_diff>
--- a/outputs/01a04c55-25c7-7382-9ab7-43cc8b274ec6/skincare-catalog-template.xlsx
+++ b/outputs/01a04c55-25c7-7382-9ab7-43cc8b274ec6/skincare-catalog-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0deb1a3e48874404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="R6ebd3bd20c6d41f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Lists" sheetId="3" r:id="R26447b2f0e5a4f46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4d4aadb6d86348be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="R83d3d99b4dbc478f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Lists" sheetId="3" r:id="R921b8b3a2af14ff3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2869,7 +2869,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68c0fd85d94944cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d2a8100de074420"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>